<commit_message>
Refactor into src/config/utils structure, add tests, CI, docs
</commit_message>
<xml_diff>
--- a/Kenya_Debt_Model.xlsx
+++ b/Kenya_Debt_Model.xlsx
@@ -356,7 +356,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="95">
+  <cellXfs count="120">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -626,6 +626,81 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="165" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -3800,7 +3875,7 @@
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B16" s="112" t="inlineStr">
         <is>
           <t>Blue fill</t>
         </is>
@@ -4124,12 +4199,12 @@
           <t>Unit</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
+      <c r="D3" s="112" t="inlineStr">
         <is>
           <t>FY22/23</t>
         </is>
       </c>
-      <c r="E3" s="7" t="inlineStr">
+      <c r="E3" s="112" t="inlineStr">
         <is>
           <t>FY23/24</t>
         </is>
@@ -5006,12 +5081,12 @@
           <t>Unit</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
+      <c r="D3" s="112" t="inlineStr">
         <is>
           <t>FY22/23</t>
         </is>
       </c>
-      <c r="E3" s="7" t="inlineStr">
+      <c r="E3" s="112" t="inlineStr">
         <is>
           <t>FY23/24</t>
         </is>
@@ -6069,12 +6144,12 @@
           <t>Category / Creditor</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="C3" s="112" t="inlineStr">
         <is>
           <t>FY22/23</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
+      <c r="D3" s="112" t="inlineStr">
         <is>
           <t>FY23/24</t>
         </is>
@@ -7316,12 +7391,12 @@
           <t>Item</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="C3" s="112" t="inlineStr">
         <is>
           <t>FY22/23</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
+      <c r="D3" s="112" t="inlineStr">
         <is>
           <t>FY23/24</t>
         </is>
@@ -7904,12 +7979,12 @@
           <t>Indicator</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="112" t="inlineStr">
         <is>
           <t>FY22/23</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="D6" s="112" t="inlineStr">
         <is>
           <t>FY23/24</t>
         </is>
@@ -9431,57 +9506,57 @@
   <sheetData>
     <row r="1" ht="8" customHeight="1"/>
     <row r="2" ht="30" customHeight="1">
-      <c r="B2" s="89" t="inlineStr">
+      <c r="B2" s="115" t="inlineStr">
         <is>
           <t>KENYA DSA MODEL — CHARTS &amp; VISUALISATIONS</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="90" t="inlineStr">
+      <c r="B4" s="116" t="inlineStr">
         <is>
           <t>Chart 1 Data — Debt/GDP vs Anchor</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="91" t="inlineStr"/>
-      <c r="C5" s="91" t="inlineStr">
+      <c r="B5" s="117" t="inlineStr"/>
+      <c r="C5" s="117" t="inlineStr">
         <is>
           <t>FY22/23</t>
         </is>
       </c>
-      <c r="D5" s="91" t="inlineStr">
+      <c r="D5" s="117" t="inlineStr">
         <is>
           <t>FY23/24</t>
         </is>
       </c>
-      <c r="E5" s="91" t="inlineStr">
+      <c r="E5" s="117" t="inlineStr">
         <is>
           <t>FY24/25</t>
         </is>
       </c>
-      <c r="F5" s="91" t="inlineStr">
+      <c r="F5" s="117" t="inlineStr">
         <is>
           <t>FY25/26</t>
         </is>
       </c>
-      <c r="G5" s="91" t="inlineStr">
+      <c r="G5" s="117" t="inlineStr">
         <is>
           <t>FY26/27</t>
         </is>
       </c>
-      <c r="H5" s="91" t="inlineStr">
+      <c r="H5" s="117" t="inlineStr">
         <is>
           <t>FY27/28</t>
         </is>
       </c>
-      <c r="I5" s="91" t="inlineStr">
+      <c r="I5" s="117" t="inlineStr">
         <is>
           <t>FY28/29</t>
         </is>
       </c>
-      <c r="J5" s="91" t="inlineStr">
+      <c r="J5" s="117" t="inlineStr">
         <is>
           <t>FY29/30</t>
         </is>
@@ -9493,28 +9568,28 @@
           <t>Debt/GDP Baseline (%)</t>
         </is>
       </c>
-      <c r="C6" s="93" t="n">
+      <c r="C6" s="118" t="n">
         <v>52.3</v>
       </c>
-      <c r="D6" s="93" t="n">
+      <c r="D6" s="118" t="n">
         <v>57.1</v>
       </c>
-      <c r="E6" s="93" t="n">
+      <c r="E6" s="118" t="n">
         <v>63.7</v>
       </c>
-      <c r="F6" s="93" t="n">
+      <c r="F6" s="118" t="n">
         <v>62.5</v>
       </c>
-      <c r="G6" s="93" t="n">
+      <c r="G6" s="118" t="n">
         <v>61</v>
       </c>
-      <c r="H6" s="93" t="n">
+      <c r="H6" s="118" t="n">
         <v>59.8</v>
       </c>
-      <c r="I6" s="93" t="n">
+      <c r="I6" s="118" t="n">
         <v>58.5</v>
       </c>
-      <c r="J6" s="93" t="n">
+      <c r="J6" s="118" t="n">
         <v>57.2</v>
       </c>
     </row>
@@ -9524,66 +9599,66 @@
           <t>55% Anchor</t>
         </is>
       </c>
-      <c r="C7" s="93" t="n">
+      <c r="C7" s="118" t="n">
         <v>55</v>
       </c>
-      <c r="D7" s="93" t="n">
+      <c r="D7" s="118" t="n">
         <v>55</v>
       </c>
-      <c r="E7" s="93" t="n">
+      <c r="E7" s="118" t="n">
         <v>55</v>
       </c>
-      <c r="F7" s="93" t="n">
+      <c r="F7" s="118" t="n">
         <v>55</v>
       </c>
-      <c r="G7" s="93" t="n">
+      <c r="G7" s="118" t="n">
         <v>55</v>
       </c>
-      <c r="H7" s="93" t="n">
+      <c r="H7" s="118" t="n">
         <v>55</v>
       </c>
-      <c r="I7" s="93" t="n">
+      <c r="I7" s="118" t="n">
         <v>55</v>
       </c>
-      <c r="J7" s="93" t="n">
+      <c r="J7" s="118" t="n">
         <v>55</v>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="90" t="inlineStr">
+      <c r="B9" s="116" t="inlineStr">
         <is>
           <t>Chart 2 Data — Scenario Fan (Debt/GDP %)</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="91" t="inlineStr"/>
-      <c r="C10" s="91" t="inlineStr">
+      <c r="B10" s="117" t="inlineStr"/>
+      <c r="C10" s="117" t="inlineStr">
         <is>
           <t>FY24/25</t>
         </is>
       </c>
-      <c r="D10" s="91" t="inlineStr">
+      <c r="D10" s="117" t="inlineStr">
         <is>
           <t>FY25/26</t>
         </is>
       </c>
-      <c r="E10" s="91" t="inlineStr">
+      <c r="E10" s="117" t="inlineStr">
         <is>
           <t>FY26/27</t>
         </is>
       </c>
-      <c r="F10" s="91" t="inlineStr">
+      <c r="F10" s="117" t="inlineStr">
         <is>
           <t>FY27/28</t>
         </is>
       </c>
-      <c r="G10" s="91" t="inlineStr">
+      <c r="G10" s="117" t="inlineStr">
         <is>
           <t>FY28/29</t>
         </is>
       </c>
-      <c r="H10" s="91" t="inlineStr">
+      <c r="H10" s="117" t="inlineStr">
         <is>
           <t>FY29/30</t>
         </is>
@@ -9595,22 +9670,22 @@
           <t>Baseline</t>
         </is>
       </c>
-      <c r="C11" s="93" t="n">
+      <c r="C11" s="118" t="n">
         <v>63.7</v>
       </c>
-      <c r="D11" s="93" t="n">
+      <c r="D11" s="118" t="n">
         <v>62.5</v>
       </c>
-      <c r="E11" s="93" t="n">
+      <c r="E11" s="118" t="n">
         <v>61</v>
       </c>
-      <c r="F11" s="93" t="n">
+      <c r="F11" s="118" t="n">
         <v>59.8</v>
       </c>
-      <c r="G11" s="93" t="n">
+      <c r="G11" s="118" t="n">
         <v>58.5</v>
       </c>
-      <c r="H11" s="93" t="n">
+      <c r="H11" s="118" t="n">
         <v>57.2</v>
       </c>
     </row>
@@ -9620,22 +9695,22 @@
           <t>Lower Growth</t>
         </is>
       </c>
-      <c r="C12" s="93" t="n">
+      <c r="C12" s="118" t="n">
         <v>63.7</v>
       </c>
-      <c r="D12" s="93" t="n">
+      <c r="D12" s="118" t="n">
         <v>66.40000000000001</v>
       </c>
-      <c r="E12" s="93" t="n">
+      <c r="E12" s="118" t="n">
         <v>66.90000000000001</v>
       </c>
-      <c r="F12" s="93" t="n">
+      <c r="F12" s="118" t="n">
         <v>67.3</v>
       </c>
-      <c r="G12" s="93" t="n">
+      <c r="G12" s="118" t="n">
         <v>67.5</v>
       </c>
-      <c r="H12" s="93" t="n">
+      <c r="H12" s="118" t="n">
         <v>67.40000000000001</v>
       </c>
     </row>
@@ -9645,22 +9720,22 @@
           <t>FX Depreciation</t>
         </is>
       </c>
-      <c r="C13" s="93" t="n">
+      <c r="C13" s="118" t="n">
         <v>63.7</v>
       </c>
-      <c r="D13" s="93" t="n">
+      <c r="D13" s="118" t="n">
         <v>69.2</v>
       </c>
-      <c r="E13" s="93" t="n">
+      <c r="E13" s="118" t="n">
         <v>67.8</v>
       </c>
-      <c r="F13" s="93" t="n">
+      <c r="F13" s="118" t="n">
         <v>65.5</v>
       </c>
-      <c r="G13" s="93" t="n">
+      <c r="G13" s="118" t="n">
         <v>63</v>
       </c>
-      <c r="H13" s="93" t="n">
+      <c r="H13" s="118" t="n">
         <v>61</v>
       </c>
     </row>
@@ -9670,22 +9745,22 @@
           <t>Interest Shock</t>
         </is>
       </c>
-      <c r="C14" s="93" t="n">
+      <c r="C14" s="118" t="n">
         <v>63.7</v>
       </c>
-      <c r="D14" s="93" t="n">
+      <c r="D14" s="118" t="n">
         <v>64</v>
       </c>
-      <c r="E14" s="93" t="n">
+      <c r="E14" s="118" t="n">
         <v>63.2</v>
       </c>
-      <c r="F14" s="93" t="n">
+      <c r="F14" s="118" t="n">
         <v>62.1</v>
       </c>
-      <c r="G14" s="93" t="n">
+      <c r="G14" s="118" t="n">
         <v>61</v>
       </c>
-      <c r="H14" s="93" t="n">
+      <c r="H14" s="118" t="n">
         <v>60</v>
       </c>
     </row>
@@ -9695,22 +9770,22 @@
           <t>Revenue Shortfall</t>
         </is>
       </c>
-      <c r="C15" s="93" t="n">
+      <c r="C15" s="118" t="n">
         <v>63.7</v>
       </c>
-      <c r="D15" s="93" t="n">
+      <c r="D15" s="118" t="n">
         <v>66.8</v>
       </c>
-      <c r="E15" s="93" t="n">
+      <c r="E15" s="118" t="n">
         <v>68.40000000000001</v>
       </c>
-      <c r="F15" s="93" t="n">
+      <c r="F15" s="118" t="n">
         <v>70.09999999999999</v>
       </c>
-      <c r="G15" s="93" t="n">
+      <c r="G15" s="118" t="n">
         <v>71.5</v>
       </c>
-      <c r="H15" s="93" t="n">
+      <c r="H15" s="118" t="n">
         <v>72.8</v>
       </c>
     </row>
@@ -9720,70 +9795,70 @@
           <t>Optimistic</t>
         </is>
       </c>
-      <c r="C16" s="93" t="n">
+      <c r="C16" s="118" t="n">
         <v>63.7</v>
       </c>
-      <c r="D16" s="93" t="n">
+      <c r="D16" s="118" t="n">
         <v>61</v>
       </c>
-      <c r="E16" s="93" t="n">
+      <c r="E16" s="118" t="n">
         <v>58.8</v>
       </c>
-      <c r="F16" s="93" t="n">
+      <c r="F16" s="118" t="n">
         <v>56.5</v>
       </c>
-      <c r="G16" s="93" t="n">
+      <c r="G16" s="118" t="n">
         <v>54.2</v>
       </c>
-      <c r="H16" s="93" t="n">
+      <c r="H16" s="118" t="n">
         <v>52</v>
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="90" t="inlineStr">
+      <c r="B18" s="116" t="inlineStr">
         <is>
           <t>Chart 3 Data — Debt Service / Revenue</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="91" t="inlineStr"/>
-      <c r="C19" s="91" t="inlineStr">
+      <c r="B19" s="117" t="inlineStr"/>
+      <c r="C19" s="117" t="inlineStr">
         <is>
           <t>FY22/23</t>
         </is>
       </c>
-      <c r="D19" s="91" t="inlineStr">
+      <c r="D19" s="117" t="inlineStr">
         <is>
           <t>FY23/24</t>
         </is>
       </c>
-      <c r="E19" s="91" t="inlineStr">
+      <c r="E19" s="117" t="inlineStr">
         <is>
           <t>FY24/25</t>
         </is>
       </c>
-      <c r="F19" s="91" t="inlineStr">
+      <c r="F19" s="117" t="inlineStr">
         <is>
           <t>FY25/26</t>
         </is>
       </c>
-      <c r="G19" s="91" t="inlineStr">
+      <c r="G19" s="117" t="inlineStr">
         <is>
           <t>FY26/27</t>
         </is>
       </c>
-      <c r="H19" s="91" t="inlineStr">
+      <c r="H19" s="117" t="inlineStr">
         <is>
           <t>FY27/28</t>
         </is>
       </c>
-      <c r="I19" s="91" t="inlineStr">
+      <c r="I19" s="117" t="inlineStr">
         <is>
           <t>FY28/29</t>
         </is>
       </c>
-      <c r="J19" s="91" t="inlineStr">
+      <c r="J19" s="117" t="inlineStr">
         <is>
           <t>FY29/30</t>
         </is>
@@ -9795,28 +9870,28 @@
           <t>DS/Revenue (%)</t>
         </is>
       </c>
-      <c r="C20" s="93" t="n">
+      <c r="C20" s="118" t="n">
         <v>47</v>
       </c>
-      <c r="D20" s="93" t="n">
+      <c r="D20" s="118" t="n">
         <v>50.2</v>
       </c>
-      <c r="E20" s="93" t="n">
+      <c r="E20" s="118" t="n">
         <v>71.2</v>
       </c>
-      <c r="F20" s="93" t="n">
+      <c r="F20" s="118" t="n">
         <v>66.5</v>
       </c>
-      <c r="G20" s="93" t="n">
+      <c r="G20" s="118" t="n">
         <v>62</v>
       </c>
-      <c r="H20" s="93" t="n">
+      <c r="H20" s="118" t="n">
         <v>58.8</v>
       </c>
-      <c r="I20" s="93" t="n">
+      <c r="I20" s="118" t="n">
         <v>55.2</v>
       </c>
-      <c r="J20" s="93" t="n">
+      <c r="J20" s="118" t="n">
         <v>52</v>
       </c>
     </row>
@@ -9826,76 +9901,76 @@
           <t>30% Threshold</t>
         </is>
       </c>
-      <c r="C21" s="93" t="n">
+      <c r="C21" s="118" t="n">
         <v>30</v>
       </c>
-      <c r="D21" s="93" t="n">
+      <c r="D21" s="118" t="n">
         <v>30</v>
       </c>
-      <c r="E21" s="93" t="n">
+      <c r="E21" s="118" t="n">
         <v>30</v>
       </c>
-      <c r="F21" s="93" t="n">
+      <c r="F21" s="118" t="n">
         <v>30</v>
       </c>
-      <c r="G21" s="93" t="n">
+      <c r="G21" s="118" t="n">
         <v>30</v>
       </c>
-      <c r="H21" s="93" t="n">
+      <c r="H21" s="118" t="n">
         <v>30</v>
       </c>
-      <c r="I21" s="93" t="n">
+      <c r="I21" s="118" t="n">
         <v>30</v>
       </c>
-      <c r="J21" s="93" t="n">
+      <c r="J21" s="118" t="n">
         <v>30</v>
       </c>
     </row>
     <row r="23">
-      <c r="B23" s="90" t="inlineStr">
+      <c r="B23" s="116" t="inlineStr">
         <is>
           <t>Chart 4 Data — Debt Composition (KES Bn)</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="91" t="inlineStr"/>
-      <c r="C24" s="91" t="inlineStr">
+      <c r="B24" s="117" t="inlineStr"/>
+      <c r="C24" s="117" t="inlineStr">
         <is>
           <t>FY22/23</t>
         </is>
       </c>
-      <c r="D24" s="91" t="inlineStr">
+      <c r="D24" s="117" t="inlineStr">
         <is>
           <t>FY23/24</t>
         </is>
       </c>
-      <c r="E24" s="91" t="inlineStr">
+      <c r="E24" s="117" t="inlineStr">
         <is>
           <t>FY24/25</t>
         </is>
       </c>
-      <c r="F24" s="91" t="inlineStr">
+      <c r="F24" s="117" t="inlineStr">
         <is>
           <t>FY25/26</t>
         </is>
       </c>
-      <c r="G24" s="91" t="inlineStr">
+      <c r="G24" s="117" t="inlineStr">
         <is>
           <t>FY26/27</t>
         </is>
       </c>
-      <c r="H24" s="91" t="inlineStr">
+      <c r="H24" s="117" t="inlineStr">
         <is>
           <t>FY27/28</t>
         </is>
       </c>
-      <c r="I24" s="91" t="inlineStr">
+      <c r="I24" s="117" t="inlineStr">
         <is>
           <t>FY28/29</t>
         </is>
       </c>
-      <c r="J24" s="91" t="inlineStr">
+      <c r="J24" s="117" t="inlineStr">
         <is>
           <t>FY29/30</t>
         </is>
@@ -9907,28 +9982,28 @@
           <t>Domestic Debt</t>
         </is>
       </c>
-      <c r="C25" s="93" t="n">
+      <c r="C25" s="118" t="n">
         <v>1300</v>
       </c>
-      <c r="D25" s="93" t="n">
+      <c r="D25" s="118" t="n">
         <v>1480</v>
       </c>
-      <c r="E25" s="93" t="n">
+      <c r="E25" s="118" t="n">
         <v>1640</v>
       </c>
-      <c r="F25" s="93" t="n">
+      <c r="F25" s="118" t="n">
         <v>1750</v>
       </c>
-      <c r="G25" s="93" t="n">
+      <c r="G25" s="118" t="n">
         <v>1830</v>
       </c>
-      <c r="H25" s="93" t="n">
+      <c r="H25" s="118" t="n">
         <v>1880</v>
       </c>
-      <c r="I25" s="93" t="n">
+      <c r="I25" s="118" t="n">
         <v>1910</v>
       </c>
-      <c r="J25" s="93" t="n">
+      <c r="J25" s="118" t="n">
         <v>1950</v>
       </c>
     </row>
@@ -9938,28 +10013,28 @@
           <t>External Debt</t>
         </is>
       </c>
-      <c r="C26" s="93" t="n">
+      <c r="C26" s="118" t="n">
         <v>4160</v>
       </c>
-      <c r="D26" s="93" t="n">
+      <c r="D26" s="118" t="n">
         <v>4510</v>
       </c>
-      <c r="E26" s="93" t="n">
+      <c r="E26" s="118" t="n">
         <v>4475</v>
       </c>
-      <c r="F26" s="93" t="n">
+      <c r="F26" s="118" t="n">
         <v>4495</v>
       </c>
-      <c r="G26" s="93" t="n">
+      <c r="G26" s="118" t="n">
         <v>4485</v>
       </c>
-      <c r="H26" s="93" t="n">
+      <c r="H26" s="118" t="n">
         <v>4475</v>
       </c>
-      <c r="I26" s="93" t="n">
+      <c r="I26" s="118" t="n">
         <v>4440</v>
       </c>
-      <c r="J26" s="93" t="n">
+      <c r="J26" s="118" t="n">
         <v>4390</v>
       </c>
     </row>
@@ -9969,50 +10044,50 @@
           <t>Guaranteed Debt</t>
         </is>
       </c>
-      <c r="C27" s="93" t="n">
+      <c r="C27" s="118" t="n">
         <v>220</v>
       </c>
-      <c r="D27" s="93" t="n">
+      <c r="D27" s="118" t="n">
         <v>209</v>
       </c>
-      <c r="E27" s="93" t="n">
+      <c r="E27" s="118" t="n">
         <v>202</v>
       </c>
-      <c r="F27" s="93" t="n">
+      <c r="F27" s="118" t="n">
         <v>189</v>
       </c>
-      <c r="G27" s="93" t="n">
+      <c r="G27" s="118" t="n">
         <v>180</v>
       </c>
-      <c r="H27" s="93" t="n">
+      <c r="H27" s="118" t="n">
         <v>173</v>
       </c>
-      <c r="I27" s="93" t="n">
+      <c r="I27" s="118" t="n">
         <v>169</v>
       </c>
-      <c r="J27" s="93" t="n">
+      <c r="J27" s="118" t="n">
         <v>165</v>
       </c>
     </row>
     <row r="35">
-      <c r="B35" s="94" t="inlineStr">
+      <c r="B35" s="119" t="inlineStr">
         <is>
           <t>Chart 1 — Debt/GDP Trend</t>
         </is>
       </c>
-      <c r="N35" s="94" t="inlineStr">
+      <c r="N35" s="119" t="inlineStr">
         <is>
           <t>Chart 2 — Scenario Fan</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="B56" s="94" t="inlineStr">
+      <c r="B56" s="119" t="inlineStr">
         <is>
           <t>Chart 3 — Debt Service / Revenue</t>
         </is>
       </c>
-      <c r="N56" s="94" t="inlineStr">
+      <c r="N56" s="119" t="inlineStr">
         <is>
           <t>Chart 4 — Debt Composition</t>
         </is>

</xml_diff>